<commit_message>
Sync generated repository state
</commit_message>
<xml_diff>
--- a/assets/downloads/sap-lead-assessment-master.xlsx
+++ b/assets/downloads/sap-lead-assessment-master.xlsx
@@ -167,7 +167,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11">
@@ -177,7 +177,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12">
@@ -188,7 +188,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.3%</t>
+          <t xml:space="preserve">38.1%</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,9 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales Processes — https://dkharlanau.github.io/labs/enterprise-context/sales-processes/</t>
+          <t xml:space="preserve">Sales Processes — https://dkharlanau.github.io/labs/enterprise-context/sales-processes/
+Sales Organizational Context &amp; Master Data — https://dkharlanau.github.io/labs/enterprise-context/sales-processes/master-data/
+Sales Lead Assessment Map — https://dkharlanau.github.io/labs/assessment/sales/</t>
         </is>
       </c>
       <c r="J2" t="n">
@@ -5899,7 +5901,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -6029,7 +6031,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -6094,7 +6096,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -6159,7 +6161,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -6224,7 +6226,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -6289,7 +6291,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle, lead-team</t>
+          <t xml:space="preserve">delivery-lifecycle, lead-team, sales-o2c</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -6354,7 +6356,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -6419,7 +6421,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -6484,7 +6486,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -6614,7 +6616,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-ams, delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -6679,7 +6681,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -6744,7 +6746,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -6809,7 +6811,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -6939,7 +6941,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -7004,7 +7006,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -7069,7 +7071,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -7134,7 +7136,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -7249,7 +7251,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -7259,12 +7261,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">sales-o2c</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle, logistics-ewm, logistics-tm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -7654,7 +7656,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, integration-cleancore, integration-deployment</t>
+          <t xml:space="preserve">sales-o2c, ai-readiness, integration-cleancore</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -8564,7 +8566,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, delivery-observability, integration-observability</t>
+          <t xml:space="preserve">sales-o2c, ai-readiness, delivery-observability</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -11749,12 +11751,12 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-ownership, integration-deployment, logistics-mdg</t>
+          <t xml:space="preserve">integration-ownership, sales-o2c, integration-deployment</t>
         </is>
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="J121" t="n">
@@ -12919,7 +12921,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-production-quality, ai-readiness, delivery-observability</t>
+          <t xml:space="preserve">logistics-production-quality, sales-o2c, ai-readiness</t>
         </is>
       </c>
       <c r="I139" t="inlineStr">
@@ -14609,7 +14611,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-observability, integration-recovery, delivery-release</t>
+          <t xml:space="preserve">sales-o2c, integration-observability, integration-recovery</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
@@ -15584,7 +15586,7 @@
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-master-data, sales-o2c, logistics-tm</t>
+          <t xml:space="preserve">sales-o2c, logistics-master-data, logistics-tm</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
@@ -18299,7 +18301,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">needs_decision</t>
+          <t xml:space="preserve">mapped</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -18309,17 +18311,17 @@
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">sales-o2c</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t xml:space="preserve">P3</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="J222" t="n">
@@ -19744,7 +19746,7 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, sales-o2c</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
@@ -20706,10 +20708,10 @@
         <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16">
@@ -21828,10 +21830,10 @@
         <v>4</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -23484,7 +23486,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -23558,7 +23560,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -23595,7 +23597,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -23632,7 +23634,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -23669,7 +23671,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -23706,7 +23708,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle, lead-team</t>
+          <t xml:space="preserve">delivery-lifecycle, lead-team, sales-o2c</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -23743,7 +23745,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -23780,7 +23782,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -23817,7 +23819,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -23891,7 +23893,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-ams, delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -23928,7 +23930,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -23965,7 +23967,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -24002,7 +24004,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -24076,7 +24078,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -24113,7 +24115,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -24150,7 +24152,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -24187,7 +24189,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle</t>
+          <t xml:space="preserve">delivery-lifecycle, sales-o2c</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -24251,17 +24253,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales</t>
+          <t xml:space="preserve">SAP Lead Assessment — Start Here</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/assessment/sales/</t>
+          <t xml:space="preserve">/labs/assessment/start-here/</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-lifecycle, logistics-ewm, logistics-tm</t>
+          <t xml:space="preserve">ai-readiness, delivery-lifecycle, delivery-testing</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -24271,7 +24273,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/assessment/sales/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/assessment/start-here/</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -24283,22 +24285,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assessment Practice</t>
+          <t xml:space="preserve">Business AI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Assessment — Start Here</t>
+          <t xml:space="preserve">Business AI Implementation Cases — Business AI Lab</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/assessment/start-here/</t>
+          <t xml:space="preserve">/labs/business-ai/cases/</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, delivery-lifecycle, delivery-testing</t>
+          <t xml:space="preserve">ai-readiness, delivery-testing, integration-observability</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -24308,7 +24310,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/assessment/start-here/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/cases/</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -24325,17 +24327,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Implementation Cases — Business AI Lab</t>
+          <t xml:space="preserve">Document-to-ERP AI Pilot — From PDF to Controlled Transaction</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/cases/</t>
+          <t xml:space="preserve">/labs/business-ai/document-to-erp-ai/</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, delivery-testing, integration-observability</t>
+          <t xml:space="preserve">integration-recovery, sales-o2c, ai-readiness</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -24345,7 +24347,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/cases/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/document-to-erp-ai/</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -24362,17 +24364,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Document-to-ERP AI Pilot — From PDF to Controlled Transaction</t>
+          <t xml:space="preserve">Business AI by Enterprise Domain — Business AI Lab</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/document-to-erp-ai/</t>
+          <t xml:space="preserve">/labs/business-ai/domains/</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-recovery, sales-o2c, ai-readiness</t>
+          <t xml:space="preserve">sales-o2c, ai-readiness, integration-cleancore</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -24382,7 +24384,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/document-to-erp-ai/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/domains/</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -24399,27 +24401,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI by Enterprise Domain — Business AI Lab</t>
+          <t xml:space="preserve">ERP Agent Gateway Pilot — Safe AI Tool Access to Enterprise Systems</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/domains/</t>
+          <t xml:space="preserve">/labs/business-ai/erp-agent-gateway/</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, integration-cleancore, integration-deployment</t>
+          <t xml:space="preserve">ai-agents-mcp, ai-security, ai-data-governance</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/domains/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/erp-agent-gateway/</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -24436,27 +24438,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">ERP Agent Gateway Pilot — Safe AI Tool Access to Enterprise Systems</t>
+          <t xml:space="preserve">Business AI Assessment Matrix — Process, Autonomy, Risk, KPI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/erp-agent-gateway/</t>
+          <t xml:space="preserve">/labs/business-ai/matrix/</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-agents-mcp, ai-security, ai-data-governance</t>
+          <t xml:space="preserve">ai-business-value, delivery-testing, lead-answer</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/erp-agent-gateway/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/matrix/</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -24473,17 +24475,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Assessment Matrix — Process, Autonomy, Risk, KPI</t>
+          <t xml:space="preserve">Business AI Graph Model — Business AI Lab</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/matrix/</t>
+          <t xml:space="preserve">/labs/business-ai/model/</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-business-value, delivery-testing, lead-answer</t>
+          <t xml:space="preserve">ai-readiness, delivery-testing, lead-answer</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -24493,7 +24495,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/matrix/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/model/</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -24510,17 +24512,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Graph Model — Business AI Lab</t>
+          <t xml:space="preserve">Open Enterprise AI Research — ERP Evidence, Safety, and Readiness</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/model/</t>
+          <t xml:space="preserve">/labs/business-ai/open-research/</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, delivery-testing, lead-answer</t>
+          <t xml:space="preserve">ai-data-governance, delivery-testing, ai-evaluation</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -24530,7 +24532,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/model/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/open-research/</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -24547,17 +24549,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Enterprise AI Research — ERP Evidence, Safety, and Readiness</t>
+          <t xml:space="preserve">Business AI Patterns — Business AI Lab</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/open-research/</t>
+          <t xml:space="preserve">/labs/business-ai/patterns/</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-data-governance, delivery-testing, ai-evaluation</t>
+          <t xml:space="preserve">integration-deployment, ai-evaluation, ai-readiness</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -24567,7 +24569,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/open-research/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/patterns/</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -24584,17 +24586,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Patterns — Business AI Lab</t>
+          <t xml:space="preserve">Open Enterprise AI Pilots — ERP, Documents, Agents, and Controls</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/patterns/</t>
+          <t xml:space="preserve">/labs/business-ai/pilots/</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-deployment, ai-evaluation, ai-readiness</t>
+          <t xml:space="preserve">ai-agents-mcp, ai-readiness, ai-data-governance</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -24604,7 +24606,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/patterns/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/pilots/</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -24621,17 +24623,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Open Enterprise AI Pilots — ERP, Documents, Agents, and Controls</t>
+          <t xml:space="preserve">Business AI Best Practices and Anti-Patterns</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/pilots/</t>
+          <t xml:space="preserve">/labs/business-ai/practices/</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-agents-mcp, ai-readiness, ai-data-governance</t>
+          <t xml:space="preserve">ai-readiness, ai-business-value, ai-evaluation</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -24641,7 +24643,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/pilots/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/practices/</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -24658,17 +24660,17 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Best Practices and Anti-Patterns</t>
+          <t xml:space="preserve">Enterprise Processes for Business AI — Business AI Lab</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/practices/</t>
+          <t xml:space="preserve">/labs/business-ai/processes/</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, ai-business-value, ai-evaluation</t>
+          <t xml:space="preserve">sales-o2c, ai-readiness, delivery-observability</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -24678,7 +24680,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/practices/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/processes/</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -24695,17 +24697,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enterprise Processes for Business AI — Business AI Lab</t>
+          <t xml:space="preserve">Business AI Scenarios — Successes, Mixed Results, Failures</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/processes/</t>
+          <t xml:space="preserve">/labs/business-ai/scenarios/</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, delivery-observability, integration-observability</t>
+          <t xml:space="preserve">delivery-testing, ai-readiness, delivery-memory</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -24715,7 +24717,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/processes/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/scenarios/</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -24732,27 +24734,27 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI Scenarios — Successes, Mixed Results, Failures</t>
+          <t xml:space="preserve">Enterprise AI Technology Landscape — Business AI Lab</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/scenarios/</t>
+          <t xml:space="preserve">/labs/business-ai/technologies/</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-testing, ai-readiness, delivery-memory</t>
+          <t xml:space="preserve">integration-cleancore, integration-deployment, integration-ownership</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/scenarios/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/technologies/</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -24764,22 +24766,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI</t>
+          <t xml:space="preserve">SAP AIF</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enterprise AI Technology Landscape — Business AI Lab</t>
+          <t xml:space="preserve">Aif</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/business-ai/technologies/</t>
+          <t xml:space="preserve">/labs/enterprise-context/aif/</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-cleancore, integration-deployment, integration-ownership</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -24789,7 +24791,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/business-ai/technologies/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/aif/</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -24801,17 +24803,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP AIF</t>
+          <t xml:space="preserve">SAP Automotive JIT/JIS</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aif</t>
+          <t xml:space="preserve">Automotive Jit</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/aif/</t>
+          <t xml:space="preserve">/labs/enterprise-context/automotive-jit/</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -24826,7 +24828,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/aif/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/automotive-jit/</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -24838,32 +24840,32 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Automotive JIT/JIS</t>
+          <t xml:space="preserve">Business AI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automotive Jit</t>
+          <t xml:space="preserve">Agents</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/automotive-jit/</t>
+          <t xml:space="preserve">/labs/enterprise-context/business-ai/agents/</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">ai-agents-mcp, delivery-cicd</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/automotive-jit/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/agents/</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -24880,12 +24882,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agents</t>
+          <t xml:space="preserve">Terminology</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/business-ai/agents/</t>
+          <t xml:space="preserve">/labs/enterprise-context/business-ai/agents/terminology/</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -24900,7 +24902,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/agents/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/agents/terminology/</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -24917,27 +24919,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminology</t>
+          <t xml:space="preserve">SAP Business AI and AI Platform Landscape — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/business-ai/agents/terminology/</t>
+          <t xml:space="preserve">/labs/enterprise-context/business-ai/</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-agents-mcp, delivery-cicd</t>
+          <t xml:space="preserve">integration-cleancore, ai-agents-mcp, delivery-release</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">P3</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/agents/terminology/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -24949,32 +24951,32 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business AI</t>
+          <t xml:space="preserve">Business Partner / CVI</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Business AI and AI Platform Landscape — Enterprise Context Lab</t>
+          <t xml:space="preserve">Business Partner</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/business-ai/</t>
+          <t xml:space="preserve">/labs/enterprise-context/business-partner/</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-cleancore, ai-agents-mcp, delivery-release</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-ai/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-partner/</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -24986,32 +24988,32 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Partner / CVI</t>
+          <t xml:space="preserve">Condition Contract Management</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Partner</t>
+          <t xml:space="preserve">Procurement</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/business-partner/</t>
+          <t xml:space="preserve">/labs/enterprise-context/condition-contract-management/procurement/</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">logistics-p2p</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/business-partner/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/condition-contract-management/procurement/</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -25028,27 +25030,27 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procurement</t>
+          <t xml:space="preserve">Sales</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/condition-contract-management/procurement/</t>
+          <t xml:space="preserve">/labs/enterprise-context/condition-contract-management/sales/</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-p2p</t>
+          <t xml:space="preserve">logistics-ewm, logistics-tm, sales-diagnostics</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/condition-contract-management/procurement/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/condition-contract-management/sales/</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -25060,32 +25062,32 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Condition Contract Management</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales</t>
+          <t xml:space="preserve">Decisions</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/condition-contract-management/sales/</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/aatp-prioritization.html</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-ewm, logistics-tm, sales-diagnostics</t>
+          <t xml:space="preserve">integration-deployment, logistics-mdg, logistics-p2p</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/condition-contract-management/sales/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/aatp-prioritization.html</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -25107,7 +25109,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/aatp-prioritization.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/account-assignment-ownership.html</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -25122,7 +25124,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/aatp-prioritization.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/account-assignment-ownership.html</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -25134,7 +25136,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP Logistics</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -25144,7 +25146,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/account-assignment-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/ai-logistics-boundary.html</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -25159,7 +25161,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/account-assignment-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ai-logistics-boundary.html</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -25171,7 +25173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Logistics</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -25181,7 +25183,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/ai-logistics-boundary.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/clean-core-extension-placement.html</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -25196,7 +25198,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ai-logistics-boundary.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/clean-core-extension-placement.html</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -25218,7 +25220,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/clean-core-extension-placement.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/confirmed-date-ownership.html</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -25233,7 +25235,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/clean-core-extension-placement.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/confirmed-date-ownership.html</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -25255,7 +25257,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/confirmed-date-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/delivery-block-ownership.html</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -25270,7 +25272,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/confirmed-date-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/delivery-block-ownership.html</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -25282,7 +25284,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP EWM</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -25292,7 +25294,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/delivery-block-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/ewm-execution-ownership.html</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -25307,7 +25309,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/delivery-block-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ewm-execution-ownership.html</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -25319,7 +25321,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP EWM</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -25329,7 +25331,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/ewm-execution-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/grir-ownership.html</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -25344,7 +25346,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ewm-execution-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/grir-ownership.html</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -25356,7 +25358,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">Integration Operations</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -25366,7 +25368,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/grir-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/idoc-api-event.html</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -25381,7 +25383,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/grir-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/idoc-api-event.html</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -25403,7 +25405,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/idoc-api-event.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/idoc-failure-ownership.html</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -25418,7 +25420,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/idoc-api-event.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/idoc-failure-ownership.html</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -25430,7 +25432,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integration Operations</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -25440,7 +25442,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/idoc-failure-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -25455,7 +25457,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/idoc-failure-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -25467,7 +25469,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP Master Data</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -25477,7 +25479,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/master-data-validation.html</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -25492,7 +25494,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/master-data-validation.html</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -25504,7 +25506,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Master Data</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -25514,7 +25516,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/master-data-validation.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/ordering-sequence-guarantees.html</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -25529,7 +25531,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/master-data-validation.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ordering-sequence-guarantees.html</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -25551,7 +25553,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/ordering-sequence-guarantees.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/po-change-impact.html</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -25566,7 +25568,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/ordering-sequence-guarantees.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/po-change-impact.html</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -25578,7 +25580,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP Pricing</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -25588,7 +25590,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/po-change-impact.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/pricing-ownership.html</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -25603,7 +25605,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/po-change-impact.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/pricing-ownership.html</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -25615,7 +25617,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Pricing</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -25625,7 +25627,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/pricing-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/retry-idempotency.html</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -25640,7 +25642,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/pricing-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/retry-idempotency.html</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -25662,7 +25664,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/retry-idempotency.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/sales-item-behavior-ownership.html</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -25677,7 +25679,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/retry-idempotency.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/sales-item-behavior-ownership.html</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -25699,7 +25701,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/sales-item-behavior-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/source-selection-ownership.html</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -25714,7 +25716,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/sales-item-behavior-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/source-selection-ownership.html</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -25736,7 +25738,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/source-selection-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/sto-vs-intercompany.html</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -25751,7 +25753,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/source-selection-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/sto-vs-intercompany.html</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -25773,7 +25775,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/sto-vs-intercompany.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/subcontracting-vs-standard-procurement.html</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -25788,7 +25790,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/sto-vs-intercompany.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/subcontracting-vs-standard-procurement.html</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -25800,7 +25802,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP Tax</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -25810,7 +25812,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/subcontracting-vs-standard-procurement.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/decisions/tax-ownership.html</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -25825,7 +25827,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/subcontracting-vs-standard-procurement.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/tax-ownership.html</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -25837,22 +25839,22 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Tax</t>
+          <t xml:space="preserve">ABAP / Extensibility</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decisions</t>
+          <t xml:space="preserve">ABAP Runtime and UI Toolkit — BAL, ALV, SALV and Fiori</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/decisions/tax-ownership.html</t>
+          <t xml:space="preserve">/labs/enterprise-context/development/toolbox/abap-runtime-ui/</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-deployment, logistics-mdg, logistics-p2p</t>
+          <t xml:space="preserve">integration-development, lead-answer, sales-billing</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -25862,7 +25864,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/decisions/tax-ownership.html</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/development/toolbox/abap-runtime-ui/</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -25879,17 +25881,17 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABAP Runtime and UI Toolkit — BAL, ALV, SALV and Fiori</t>
+          <t xml:space="preserve">SAP Development Toolbox — Frameworks, Quality and Delivery</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/development/toolbox/abap-runtime-ui/</t>
+          <t xml:space="preserve">/labs/enterprise-context/development/toolbox/</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-development, lead-answer, sales-billing</t>
+          <t xml:space="preserve">ai-data-governance, delivery-cicd, delivery-lifecycle</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -25899,7 +25901,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/development/toolbox/abap-runtime-ui/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/development/toolbox/</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -25911,22 +25913,22 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">ABAP / Extensibility</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Development Toolbox — Frameworks, Quality and Delivery</t>
+          <t xml:space="preserve">Enterprise Business Domains — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/development/toolbox/</t>
+          <t xml:space="preserve">/labs/enterprise-context/domains/</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-data-governance, delivery-cicd, delivery-lifecycle</t>
+          <t xml:space="preserve">integration-ownership, sales-o2c, integration-deployment</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -25936,7 +25938,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/development/toolbox/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/domains/</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -25948,22 +25950,22 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP EWM</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enterprise Business Domains — Enterprise Context Lab</t>
+          <t xml:space="preserve">Automation</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/domains/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/automation/</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-ownership, integration-deployment, logistics-mdg</t>
+          <t xml:space="preserve">ai-data-governance, logistics-ewm</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -25973,7 +25975,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/domains/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/automation/</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -25990,27 +25992,27 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automation</t>
+          <t xml:space="preserve">Controls</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/automation/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/controls/</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-data-governance, logistics-ewm</t>
+          <t xml:space="preserve">ai-readiness, logistics-ewm</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/automation/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/controls/</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -26027,27 +26029,27 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controls</t>
+          <t xml:space="preserve">Domains</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/controls/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/domains/</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-readiness, logistics-ewm</t>
+          <t xml:space="preserve">logistics-ewm</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/controls/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/domains/</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -26064,12 +26066,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Domains</t>
+          <t xml:space="preserve">Handling Units Packing</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/domains/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/handling-units-packing/</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -26084,7 +26086,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/domains/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/handling-units-packing/</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -26101,27 +26103,27 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handling Units Packing</t>
+          <t xml:space="preserve">Integrations</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/handling-units-packing/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/integrations/</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-ewm</t>
+          <t xml:space="preserve">integration-patterns, logistics-ewm</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/handling-units-packing/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/integrations/</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -26138,17 +26140,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrations</t>
+          <t xml:space="preserve">Interfaces</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/integrations/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/interfaces/</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns, logistics-ewm</t>
+          <t xml:space="preserve">delivery-testing, logistics-ewm</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -26158,7 +26160,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/integrations/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/interfaces/</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -26175,27 +26177,27 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interfaces</t>
+          <t xml:space="preserve">Mobility</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/interfaces/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/mobility/</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-testing, logistics-ewm</t>
+          <t xml:space="preserve">logistics-ewm</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/interfaces/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/mobility/</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -26212,12 +26214,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mobility</t>
+          <t xml:space="preserve">Objects</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/mobility/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/objects/</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -26232,7 +26234,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/mobility/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/objects/</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -26249,12 +26251,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Objects</t>
+          <t xml:space="preserve">Scanners</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/objects/</t>
+          <t xml:space="preserve">/labs/enterprise-context/ewm/scanners/</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -26269,7 +26271,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/objects/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/scanners/</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -26281,22 +26283,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP EWM</t>
+          <t xml:space="preserve">SAP Logistics</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scanners</t>
+          <t xml:space="preserve">Finance Logistics</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/ewm/scanners/</t>
+          <t xml:space="preserve">/labs/enterprise-context/finance-logistics/</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-ewm</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -26306,7 +26308,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/ewm/scanners/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/finance-logistics/</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -26318,32 +26320,32 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Logistics</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finance Logistics</t>
+          <t xml:space="preserve">BRFplus, AIF and ISLM — Decision, Recovery and AI Lifecycle</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/finance-logistics/</t>
+          <t xml:space="preserve">/labs/enterprise-context/frameworks/</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-ams, delivery-cicd, integration-cleancore</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/finance-logistics/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/frameworks/</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -26360,17 +26362,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">BRFplus, AIF and ISLM — Decision, Recovery and AI Lifecycle</t>
+          <t xml:space="preserve">Enterprise Context Lab — Process, Data, Rules and AI Reasoning</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/frameworks/</t>
+          <t xml:space="preserve">/labs/enterprise-context/</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, delivery-cicd, integration-cleancore</t>
+          <t xml:space="preserve">integration-ownership, delivery-testing, integration-patterns</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -26380,7 +26382,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/frameworks/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -26397,17 +26399,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enterprise Context Lab — Process, Data, Rules and AI Reasoning</t>
+          <t xml:space="preserve">SAP Industry Solutions — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/</t>
+          <t xml:space="preserve">/labs/enterprise-context/industries/</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-ownership, delivery-testing, integration-patterns</t>
+          <t xml:space="preserve">logistics-production-quality, sales-o2c, ai-readiness</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -26417,7 +26419,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/industries/</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -26429,22 +26431,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">Integration Architecture</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Industry Solutions — Enterprise Context Lab</t>
+          <t xml:space="preserve">Data Migration</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/industries/</t>
+          <t xml:space="preserve">/labs/enterprise-context/integrations/data-migration/</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-production-quality, ai-readiness, delivery-observability</t>
+          <t xml:space="preserve">integration-patterns</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -26454,7 +26456,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/industries/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/integrations/data-migration/</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -26466,32 +26468,32 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integration Architecture</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Data Migration</t>
+          <t xml:space="preserve">Iot Devices</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/integrations/data-migration/</t>
+          <t xml:space="preserve">/labs/enterprise-context/iot-devices/</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/integrations/data-migration/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/iot-devices/</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -26503,32 +26505,32 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP MDG / DRF</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iot Devices</t>
+          <t xml:space="preserve">SAP MDG Solution Architecture — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/iot-devices/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/architecture/</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integration-recovery, logistics-mdg, ai-data-governance</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/iot-devices/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/architecture/</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -26545,17 +26547,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Solution Architecture — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Build &amp; Runtime Anatomy — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/architecture/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/build-runtime/</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-recovery, logistics-mdg, ai-data-governance</t>
+          <t xml:space="preserve">delivery-cicd, lead-decision, ai-business-value</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -26565,7 +26567,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/architecture/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/build-runtime/</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -26582,17 +26584,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Build &amp; Runtime Anatomy — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Data Model Engineering — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/build-runtime/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/data-model/engineering/</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-cicd, lead-decision, ai-business-value</t>
+          <t xml:space="preserve">logistics-mdg, delivery-testing, ai-readiness</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -26602,7 +26604,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/build-runtime/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/data-model/engineering/</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -26619,17 +26621,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Data Model Engineering — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Data Model Anatomy — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/data-model/engineering/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/data-model/</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, delivery-testing, ai-readiness</t>
+          <t xml:space="preserve">logistics-mdg, integration-deployment, ai-readiness</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -26639,7 +26641,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/data-model/engineering/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/data-model/</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -26656,27 +26658,27 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Data Model Anatomy — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Deployment Options — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/data-model/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/deployments/</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, integration-deployment, ai-readiness</t>
+          <t xml:space="preserve">integration-deployment, lead-decision, integration-cleancore</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/data-model/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/deployments/</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -26688,32 +26690,32 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG / DRF</t>
+          <t xml:space="preserve">Business Partner / CVI</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Deployment Options — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Business Partner Entity Map — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/deployments/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/domains/business-partner/entity-map/</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-deployment, lead-decision, integration-cleancore</t>
+          <t xml:space="preserve">sales-o2c, integration-observability, integration-recovery</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/deployments/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/domains/business-partner/entity-map/</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -26725,32 +26727,32 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Business Partner / CVI</t>
+          <t xml:space="preserve">SAP MDG / DRF</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Business Partner Entity Map — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Material Entity Map — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/domains/business-partner/entity-map/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/domains/material/entity-map/</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-observability, integration-recovery, delivery-release</t>
+          <t xml:space="preserve">logistics-mdg, integration-observability, integration-ownership</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/domains/business-partner/entity-map/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/domains/material/entity-map/</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -26767,27 +26769,27 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Material Entity Map — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Extension Matrix — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/domains/material/entity-map/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/extensions/</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, integration-observability, integration-ownership</t>
+          <t xml:space="preserve">integration-cleancore, integration-deployment, delivery-testing</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/domains/material/entity-map/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/extensions/</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -26804,17 +26806,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Extension Matrix — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG BRFplus Rule Catalog — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/extensions/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/governance-engine/brfplus-rules/</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-cleancore, integration-deployment, delivery-testing</t>
+          <t xml:space="preserve">logistics-mdg, integration-deployment, integration-recovery</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -26824,7 +26826,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/extensions/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/governance-engine/brfplus-rules/</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -26841,17 +26843,17 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG BRFplus Rule Catalog — Enterprise Context Lab</t>
+          <t xml:space="preserve">MDG Attribute to Process Impact — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/governance-engine/brfplus-rules/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/impact/</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, integration-deployment, integration-recovery</t>
+          <t xml:space="preserve">sales-o2c, delivery-testing, integration-ownership</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -26861,7 +26863,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/governance-engine/brfplus-rules/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/impact/</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -26878,27 +26880,27 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDG Attribute to Process Impact — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Implementation and Presales Guide — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/impact/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/implementation/</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">sales-o2c, delivery-testing, integration-ownership</t>
+          <t xml:space="preserve">logistics-mdg, integration-deployment, integration-ownership</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/impact/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/implementation/</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -26915,27 +26917,27 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Implementation and Presales Guide — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Interface Contracts — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/implementation/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/interfaces/</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, integration-deployment, integration-ownership</t>
+          <t xml:space="preserve">integration-patterns, integration-recovery, logistics-master-data</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/implementation/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/interfaces/</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -26952,17 +26954,17 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Interface Contracts — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Lineage &amp; Provenance — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/interfaces/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/lineage/</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns, integration-recovery, logistics-master-data</t>
+          <t xml:space="preserve">logistics-mdg, ai-business-value, ai-data-governance</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -26972,7 +26974,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/interfaces/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/lineage/</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -26984,22 +26986,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG / DRF</t>
+          <t xml:space="preserve">SAP Logistics</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Lineage &amp; Provenance — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Logistics End-to-End Cases — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/lineage/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/logistics/cases/</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, ai-business-value, ai-data-governance</t>
+          <t xml:space="preserve">logistics-tm, delivery-lifecycle, logistics-ewm</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -27009,7 +27011,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/lineage/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/logistics/cases/</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -27026,17 +27028,17 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Logistics End-to-End Cases — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG for Logistics — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/logistics/cases/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/logistics/</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-tm, delivery-lifecycle, logistics-ewm</t>
+          <t xml:space="preserve">sales-o2c, logistics-master-data, logistics-tm</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -27046,7 +27048,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/logistics/cases/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/logistics/</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -27058,22 +27060,22 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Logistics</t>
+          <t xml:space="preserve">SAP MDG / DRF</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG for Logistics — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Migration &amp; Load Strategy — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/logistics/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/migration/</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-master-data, sales-o2c, logistics-tm</t>
+          <t xml:space="preserve">delivery-release, ai-readiness, delivery-testing</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -27083,7 +27085,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/logistics/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/migration/</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -27100,17 +27102,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Migration &amp; Load Strategy — Enterprise Context Lab</t>
+          <t xml:space="preserve">MDG Ownership and Federation — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/migration/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/ownership/</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-release, ai-readiness, delivery-testing</t>
+          <t xml:space="preserve">logistics-p2p, ai-readiness, logistics-master-data</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -27120,7 +27122,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/migration/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/ownership/</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -27137,27 +27139,27 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDG Ownership and Federation — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Governance Processes and Tools — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/ownership/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/processes/</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-p2p, ai-readiness, logistics-master-data</t>
+          <t xml:space="preserve">logistics-mdg, ai-data-governance, ai-agents-mcp</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P3</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/ownership/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/processes/</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -27174,27 +27176,27 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Governance Processes and Tools — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Assessment Reasoning — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/processes/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/reasoning/</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, ai-data-governance, ai-agents-mcp</t>
+          <t xml:space="preserve">delivery-testing, delivery-lifecycle, ai-agents-mcp</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">P3</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/processes/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/reasoning/</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -27211,17 +27213,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Assessment Reasoning — Enterprise Context Lab</t>
+          <t xml:space="preserve">SAP MDG Synthetic Material Scenario — Enterprise Context Lab</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/reasoning/</t>
+          <t xml:space="preserve">/labs/enterprise-context/mdg/scenario/</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-testing, delivery-lifecycle, ai-agents-mcp</t>
+          <t xml:space="preserve">logistics-mdg, integration-ownership, logistics-master-data</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -27231,7 +27233,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/reasoning/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/scenario/</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -27243,32 +27245,32 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG / DRF</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP MDG Synthetic Material Scenario — Enterprise Context Lab</t>
+          <t xml:space="preserve">Enterprise Context Lab — Model and Authoring Contract</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/mdg/scenario/</t>
+          <t xml:space="preserve">/labs/enterprise-context/model/</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg, integration-ownership, logistics-master-data</t>
+          <t xml:space="preserve">ai-data-governance, ai-retrieval, delivery-cicd</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/mdg/scenario/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/model/</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -27280,32 +27282,32 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">SAP Pricing</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enterprise Context Lab — Model and Authoring Contract</t>
+          <t xml:space="preserve">Anatomy</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/model/</t>
+          <t xml:space="preserve">/labs/enterprise-context/pricing/anatomy/</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-data-governance, ai-retrieval, delivery-cicd</t>
+          <t xml:space="preserve">sales-pricing</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/model/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/anatomy/</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -27322,12 +27324,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anatomy</t>
+          <t xml:space="preserve">Casebook</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/pricing/anatomy/</t>
+          <t xml:space="preserve">/labs/enterprise-context/pricing/casebook/</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -27342,7 +27344,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/anatomy/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/casebook/</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -27359,17 +27361,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Casebook</t>
+          <t xml:space="preserve">Configuration</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/pricing/casebook/</t>
+          <t xml:space="preserve">/labs/enterprise-context/pricing/configuration/</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t xml:space="preserve">sales-pricing</t>
+          <t xml:space="preserve">sales-pricing, delivery-testing, integration-development</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -27379,7 +27381,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/casebook/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/configuration/</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -27396,17 +27398,17 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Configuration</t>
+          <t xml:space="preserve">Operations</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/pricing/configuration/</t>
+          <t xml:space="preserve">/labs/enterprise-context/pricing/operations/</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t xml:space="preserve">sales-pricing, delivery-testing, integration-development</t>
+          <t xml:space="preserve">delivery-ams, integration-deployment, integration-recovery</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -27416,7 +27418,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/configuration/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/operations/</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -27433,17 +27435,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operations</t>
+          <t xml:space="preserve">Scenarios</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/pricing/operations/</t>
+          <t xml:space="preserve">/labs/enterprise-context/pricing/scenarios/</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, integration-deployment, integration-recovery</t>
+          <t xml:space="preserve">sales-pricing</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -27453,7 +27455,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/operations/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/scenarios/</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -27465,22 +27467,22 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Pricing</t>
+          <t xml:space="preserve">Other / Cross-domain</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scenarios</t>
+          <t xml:space="preserve">SAP S/4HANA 2025 Release Readiness Playbook</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/pricing/scenarios/</t>
+          <t xml:space="preserve">/labs/enterprise-context/release-readiness/</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t xml:space="preserve">sales-pricing</t>
+          <t xml:space="preserve">ai-evaluation, delivery-lifecycle, delivery-release</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -27490,7 +27492,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/pricing/scenarios/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/release-readiness/</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -27502,32 +27504,32 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other / Cross-domain</t>
+          <t xml:space="preserve">Analytics / Observability</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP S/4HANA 2025 Release Readiness Playbook</t>
+          <t xml:space="preserve">Sales Analytics</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/release-readiness/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-analytics/</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">ai-evaluation, delivery-lifecycle, delivery-release</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/release-readiness/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-analytics/</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -27539,17 +27541,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analytics / Observability</t>
+          <t xml:space="preserve">SAP Sales / SD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales Analytics</t>
+          <t xml:space="preserve">Sales Order</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-analytics/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-order/</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -27564,7 +27566,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-analytics/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-order/</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -27581,12 +27583,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sales Order</t>
+          <t xml:space="preserve">Control Plane</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-order/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/control-plane/</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -27601,7 +27603,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-order/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/control-plane/</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -27618,12 +27620,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control Plane</t>
+          <t xml:space="preserve">Returns Claims</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/control-plane/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/control-plane/returns-claims/</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -27638,7 +27640,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/control-plane/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/control-plane/returns-claims/</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -27655,27 +27657,27 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Returns Claims</t>
+          <t xml:space="preserve">Coverage</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/control-plane/returns-claims/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/coverage/</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">delivery-testing, lead-evidence, lead-readiness</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/control-plane/returns-claims/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/coverage/</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -27687,22 +27689,22 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Sales / SD</t>
+          <t xml:space="preserve">Integration Architecture</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coverage</t>
+          <t xml:space="preserve">Integrations</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/coverage/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/integrations/</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-testing, lead-evidence, lead-readiness</t>
+          <t xml:space="preserve">integration-patterns</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -27712,7 +27714,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/coverage/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/integrations/</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -27724,32 +27726,32 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integration Architecture</t>
+          <t xml:space="preserve">SAP Sales / SD</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrations</t>
+          <t xml:space="preserve">Derivation</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/integrations/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/mechanisms/derivation/</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/integrations/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/mechanisms/derivation/</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -27761,32 +27763,32 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Master Data</t>
+          <t xml:space="preserve">SAP Sales / SD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Master Data</t>
+          <t xml:space="preserve">Mechanisms</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/master-data/</t>
+          <t xml:space="preserve">/labs/enterprise-context/sales-processes/mechanisms/</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-mdg</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t xml:space="preserve">P3</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/master-data/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/mechanisms/</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -27798,17 +27800,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Sales / SD</t>
+          <t xml:space="preserve">SAP Tax</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Derivation</t>
+          <t xml:space="preserve">Tax</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/mechanisms/derivation/</t>
+          <t xml:space="preserve">/labs/enterprise-context/tax/</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -27823,7 +27825,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/mechanisms/derivation/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/tax/</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -27835,17 +27837,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Sales / SD</t>
+          <t xml:space="preserve">SAP TM</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mechanisms</t>
+          <t xml:space="preserve">Charges</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/sales-processes/mechanisms/</t>
+          <t xml:space="preserve">/labs/enterprise-context/transportation-management/charges/</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -27860,7 +27862,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/sales-processes/mechanisms/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/charges/</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -27872,32 +27874,32 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Tax</t>
+          <t xml:space="preserve">Integration Architecture</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tax</t>
+          <t xml:space="preserve">Integrations</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/tax/</t>
+          <t xml:space="preserve">/labs/enterprise-context/transportation-management/integrations/</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">integration-patterns</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/tax/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/integrations/</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -27914,17 +27916,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charges</t>
+          <t xml:space="preserve">Planning</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/transportation-management/charges/</t>
+          <t xml:space="preserve">/labs/enterprise-context/transportation-management/planning/</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">logistics-tm</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -27934,7 +27936,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/charges/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/planning/</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -27946,22 +27948,22 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integration Architecture</t>
+          <t xml:space="preserve">Assessment Practice</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrations</t>
+          <t xml:space="preserve">Labs — SAP Enterprise, Assurance, AI, Interview and Assessment</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/transportation-management/integrations/</t>
+          <t xml:space="preserve">/labs/</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t xml:space="preserve">integration-patterns</t>
+          <t xml:space="preserve">delivery-ams, delivery-memory, delivery-testing</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -27971,7 +27973,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/integrations/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -27983,32 +27985,32 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP TM</t>
+          <t xml:space="preserve">Interview Readiness</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planning</t>
+          <t xml:space="preserve">SAP Lead Interview Readiness — Practical Preparation Lab</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/enterprise-context/transportation-management/planning/</t>
+          <t xml:space="preserve">/labs/interview-readiness/</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-tm</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, sales-shipping</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t xml:space="preserve">P2</t>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/enterprise-context/transportation-management/planning/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -28020,22 +28022,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Assessment Practice</t>
+          <t xml:space="preserve">Interview Readiness</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Labs — SAP Enterprise, Assurance, AI, Interview and Assessment</t>
+          <t xml:space="preserve">SAP Lead Interview Practice — 12-Question Interview Mode</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/</t>
+          <t xml:space="preserve">/labs/interview-readiness/practice/</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, delivery-memory, delivery-testing</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, sales-o2c</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -28045,7 +28047,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/practice/</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -28062,17 +28064,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Readiness — Practical Preparation Lab</t>
+          <t xml:space="preserve">SAP Lead Interview Progress — Readiness and Weak Areas</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/</t>
+          <t xml:space="preserve">/labs/interview-readiness/progress/</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, sales-shipping</t>
+          <t xml:space="preserve">lead-evidence, delivery-testing, ai-readiness</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -28082,7 +28084,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/progress/</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -28099,17 +28101,17 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Practice — 12-Question Interview Mode</t>
+          <t xml:space="preserve">SAP Lead Interview Questions — 42 Skills, 168 Questions</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/practice/</t>
+          <t xml:space="preserve">/labs/interview-readiness/questions/</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
+          <t xml:space="preserve">logistics-tm, delivery-ams, integration-ownership</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -28119,7 +28121,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/practice/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/questions/</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -28136,17 +28138,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Progress — Readiness and Weak Areas</t>
+          <t xml:space="preserve">SAP Lead Career Roadmap — Skills, Labs, Evidence, Practice</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/progress/</t>
+          <t xml:space="preserve">/labs/interview-readiness/roadmap/</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t xml:space="preserve">lead-evidence, delivery-testing, ai-readiness</t>
+          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -28156,7 +28158,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/progress/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/roadmap/</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -28173,17 +28175,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Interview Questions — 42 Skills, 168 Questions</t>
+          <t xml:space="preserve">SAP Interview Story Bank — Projects, Decisions, Failures, Results</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/questions/</t>
+          <t xml:space="preserve">/labs/interview-readiness/stories/</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">logistics-tm, delivery-ams, integration-ownership</t>
+          <t xml:space="preserve">lead-evidence, integration-deployment, ai-agents-mcp</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -28193,7 +28195,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/questions/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/stories/</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -28205,32 +28207,32 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interview Readiness</t>
+          <t xml:space="preserve">Reusable Data Procedures</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Lead Career Roadmap — Skills, Labs, Evidence, Practice</t>
+          <t xml:space="preserve">Reusable Data Procedures</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/roadmap/</t>
+          <t xml:space="preserve">/labs/reusable-data-procedures/</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t xml:space="preserve">delivery-ams, logistics-tm, delivery-lifecycle</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t xml:space="preserve">P1</t>
+          <t xml:space="preserve">P2</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/roadmap/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/reusable-data-procedures/</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -28242,22 +28244,22 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interview Readiness</t>
+          <t xml:space="preserve">Tooling / Roadmap</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAP Interview Story Bank — Projects, Decisions, Failures, Results</t>
+          <t xml:space="preserve">Tool Roadmap — Portable Enterprise Tools</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t xml:space="preserve">/labs/interview-readiness/stories/</t>
+          <t xml:space="preserve">/labs/tool-roadmap/</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t xml:space="preserve">lead-evidence, integration-deployment, ai-agents-mcp</t>
+          <t xml:space="preserve">delivery-testing, ai-agents-mcp, ai-data-governance</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
@@ -28267,7 +28269,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/interview-readiness/stories/</t>
+          <t xml:space="preserve">https://dkharlanau.github.io/labs/tool-roadmap/</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -28276,82 +28278,8 @@
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reusable Data Procedures</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reusable Data Procedures</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">/labs/reusable-data-procedures/</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P2</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/reusable-data-procedures/</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tooling / Roadmap</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tool Roadmap — Portable Enterprise Tools</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">/labs/tool-roadmap/</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">delivery-testing, ai-agents-mcp, ai-data-governance</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">P1</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://dkharlanau.github.io/labs/tool-roadmap/</t>
-        </is>
-      </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G159"/>
+  <autoFilter ref="A1:G157"/>
 </worksheet>
 </file>
 

</xml_diff>